<commit_message>
Add GLASS normalization analysis
</commit_message>
<xml_diff>
--- a/archive/legacy_assets/predicted_SI.xlsx
+++ b/archive/legacy_assets/predicted_SI.xlsx
@@ -172,10 +172,10 @@
     <t>Oxazolidinones</t>
   </si>
   <si>
+    <t>yes</t>
+  </si>
+  <si>
     <t>no</t>
-  </si>
-  <si>
-    <t>yes</t>
   </si>
 </sst>
 </file>
@@ -626,7 +626,7 @@
         <v>1.183719002926647</v>
       </c>
       <c r="I3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="J3">
         <v>9.071585984706237</v>
@@ -658,7 +658,7 @@
         <v>1.002354953010338</v>
       </c>
       <c r="I4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="J4">
         <v>11.95780118076588</v>
@@ -690,7 +690,7 @@
         <v>1.101965783942812</v>
       </c>
       <c r="I5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="J5">
         <v>20.58756240828968</v>
@@ -754,7 +754,7 @@
         <v>0.9549592046414992</v>
       </c>
       <c r="I7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J7">
         <v>17.37314067381907</v>
@@ -786,7 +786,7 @@
         <v>1.072414562207262</v>
       </c>
       <c r="I8" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J8">
         <v>20.50807269882524</v>
@@ -850,7 +850,7 @@
         <v>0.8313655914345222</v>
       </c>
       <c r="I10" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J10">
         <v>15.07591724190151</v>
@@ -882,7 +882,7 @@
         <v>1.004094691773939</v>
       </c>
       <c r="I11" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="J11">
         <v>10.10437676892359</v>
@@ -914,7 +914,7 @@
         <v>0.9607544889622261</v>
       </c>
       <c r="I12" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J12">
         <v>8.091026715448415</v>
@@ -978,7 +978,7 @@
         <v>0.8074855164848718</v>
       </c>
       <c r="I14" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J14">
         <v>8.606093393731701</v>
@@ -1010,7 +1010,7 @@
         <v>0.8109736139487409</v>
       </c>
       <c r="I15" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J15">
         <v>12.79660437093753</v>
@@ -1042,7 +1042,7 @@
         <v>0.725968350096911</v>
       </c>
       <c r="I16" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J16">
         <v>8.120475123713844</v>
@@ -1106,7 +1106,7 @@
         <v>0.6496044852505278</v>
       </c>
       <c r="I18" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J18">
         <v>12.74571639444505</v>
@@ -1170,7 +1170,7 @@
         <v>0.648211080546478</v>
       </c>
       <c r="I20" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J20">
         <v>10.02441052926776</v>
@@ -1202,7 +1202,7 @@
         <v>0.6670010548273044</v>
       </c>
       <c r="I21" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="J21">
         <v>11.91071367370867</v>
@@ -1266,7 +1266,7 @@
         <v>0.6595287627412922</v>
       </c>
       <c r="I23" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J23">
         <v>24.87701442286552</v>
@@ -1298,7 +1298,7 @@
         <v>0.7818511801661132</v>
       </c>
       <c r="I24" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J24">
         <v>8.772103055789852</v>
@@ -1330,7 +1330,7 @@
         <v>0.778615562341779</v>
       </c>
       <c r="I25" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J25">
         <v>7.859441451082082</v>
@@ -1362,7 +1362,7 @@
         <v>0.7410264912224118</v>
       </c>
       <c r="I26" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="J26">
         <v>4.382943702710341</v>
@@ -1426,7 +1426,7 @@
         <v>0.6466201601316135</v>
       </c>
       <c r="I28" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J28">
         <v>14.24201271075685</v>
@@ -1458,7 +1458,7 @@
         <v>0.7561400021450257</v>
       </c>
       <c r="I29" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="J29">
         <v>14.51312263708803</v>
@@ -1490,7 +1490,7 @@
         <v>0.5657751756892995</v>
       </c>
       <c r="I30" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J30">
         <v>16.28469831565101</v>
@@ -1522,7 +1522,7 @@
         <v>0.4887199442023433</v>
       </c>
       <c r="I31" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="J31">
         <v>23.95950368535706</v>
@@ -1554,7 +1554,7 @@
         <v>0.5389104496358017</v>
       </c>
       <c r="I32" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J32">
         <v>16.79577108345717</v>
@@ -1586,7 +1586,7 @@
         <v>0.7908885539092194</v>
       </c>
       <c r="I33" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J33">
         <v>5.915743582118907</v>
@@ -1618,7 +1618,7 @@
         <v>0.5052771290170388</v>
       </c>
       <c r="I34" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J34">
         <v>11.15986825894109</v>
@@ -1746,7 +1746,7 @@
         <v>0.5826070689387459</v>
       </c>
       <c r="I38" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J38">
         <v>13.92673290562042</v>
@@ -1778,7 +1778,7 @@
         <v>0.6142311679839063</v>
       </c>
       <c r="I39" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="J39">
         <v>7.241672071835522</v>
@@ -1810,7 +1810,7 @@
         <v>0.3605213135780032</v>
       </c>
       <c r="I40" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J40">
         <v>9.405743123243324</v>
@@ -1874,7 +1874,7 @@
         <v>0.5060540892806709</v>
       </c>
       <c r="I42" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J42">
         <v>20.88899679499637</v>
@@ -1906,7 +1906,7 @@
         <v>0.3447164054891756</v>
       </c>
       <c r="I43" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J43">
         <v>19.30524576171661</v>
@@ -1970,7 +1970,7 @@
         <v>0.427074393790505</v>
       </c>
       <c r="I45" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J45">
         <v>13.19879367792396</v>
@@ -2002,7 +2002,7 @@
         <v>0.5214379594993712</v>
       </c>
       <c r="I46" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J46">
         <v>24.13876221942635</v>
@@ -2034,7 +2034,7 @@
         <v>0.5086773189739302</v>
       </c>
       <c r="I47" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J47">
         <v>16.93110445587214</v>
@@ -2066,7 +2066,7 @@
         <v>0.5134911045201391</v>
       </c>
       <c r="I48" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J48">
         <v>15.07270921511292</v>
@@ -2098,7 +2098,7 @@
         <v>0.341329375622631</v>
       </c>
       <c r="I49" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J49">
         <v>17.3435312125895</v>
@@ -2130,7 +2130,7 @@
         <v>0.292009319904533</v>
       </c>
       <c r="I50" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J50">
         <v>13.53437292203027</v>
@@ -2194,7 +2194,7 @@
         <v>0.3263571077129876</v>
       </c>
       <c r="I52" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J52">
         <v>9.43145036694629</v>
@@ -2226,7 +2226,7 @@
         <v>0.3897098508267349</v>
       </c>
       <c r="I53" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J53">
         <v>12.41451650350251</v>
@@ -2258,7 +2258,7 @@
         <v>0.5331781523858607</v>
       </c>
       <c r="I54" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J54">
         <v>15.90327209494377</v>
@@ -2290,7 +2290,7 @@
         <v>0.5088089694801923</v>
       </c>
       <c r="I55" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J55">
         <v>18.32872261437137</v>
@@ -2322,7 +2322,7 @@
         <v>0.5134988472317312</v>
       </c>
       <c r="I56" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J56">
         <v>11.83015226299159</v>
@@ -2354,7 +2354,7 @@
         <v>0.2727968421847911</v>
       </c>
       <c r="I57" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J57">
         <v>18.46621535578246</v>
@@ -2418,7 +2418,7 @@
         <v>0.5024493695731933</v>
       </c>
       <c r="I59" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J59">
         <v>14.10027015415705</v>
@@ -2450,7 +2450,7 @@
         <v>0.2032192238970947</v>
       </c>
       <c r="I60" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J60">
         <v>21.48445873543648</v>
@@ -2482,7 +2482,7 @@
         <v>0.4806698547503252</v>
       </c>
       <c r="I61" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J61">
         <v>22.02672963143239</v>
@@ -2514,7 +2514,7 @@
         <v>0.3105255081320208</v>
       </c>
       <c r="I62" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J62">
         <v>15.55108477810051</v>
@@ -2546,7 +2546,7 @@
         <v>0.5248496955731041</v>
       </c>
       <c r="I63" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J63">
         <v>21.64110764285963</v>
@@ -2610,7 +2610,7 @@
         <v>0.3892267651139838</v>
       </c>
       <c r="I65" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J65">
         <v>13.11248207792986</v>
@@ -2706,7 +2706,7 @@
         <v>0.2474241836001487</v>
       </c>
       <c r="I68" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J68">
         <v>11.56036807350337</v>
@@ -2770,7 +2770,7 @@
         <v>0.4332994565565464</v>
       </c>
       <c r="I70" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J70">
         <v>23.78244461515768</v>
@@ -2802,7 +2802,7 @@
         <v>0.4485706766248951</v>
       </c>
       <c r="I71" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J71">
         <v>14.91991941229707</v>
@@ -2834,7 +2834,7 @@
         <v>0.4771989178119607</v>
       </c>
       <c r="I72" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J72">
         <v>17.36455934537124</v>
@@ -2866,7 +2866,7 @@
         <v>0.2681090566240896</v>
       </c>
       <c r="I73" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J73">
         <v>20.31634113418007</v>
@@ -2898,7 +2898,7 @@
         <v>0.352298078666452</v>
       </c>
       <c r="I74" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J74">
         <v>15.93342650708624</v>
@@ -2962,7 +2962,7 @@
         <v>0.1592268907630912</v>
       </c>
       <c r="I76" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J76">
         <v>20.82430157481807</v>
@@ -3026,7 +3026,7 @@
         <v>0.124020270960528</v>
       </c>
       <c r="I78" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J78">
         <v>20.96651980317871</v>
@@ -3058,7 +3058,7 @@
         <v>0.2678481730624225</v>
       </c>
       <c r="I79" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J79">
         <v>24.49258294760917</v>
@@ -3090,7 +3090,7 @@
         <v>0.3132827272867045</v>
       </c>
       <c r="I80" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J80">
         <v>17.28943877287773</v>
@@ -3122,7 +3122,7 @@
         <v>0.3444331189228456</v>
       </c>
       <c r="I81" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J81">
         <v>20.46178265347313</v>
@@ -3154,7 +3154,7 @@
         <v>0.3071417659357354</v>
       </c>
       <c r="I82" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J82">
         <v>17.91631842151344</v>
@@ -3186,7 +3186,7 @@
         <v>-0.07191773300934057</v>
       </c>
       <c r="I83" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J83">
         <v>18.55981365758918</v>
@@ -3218,7 +3218,7 @@
         <v>0.0005005074335733273</v>
       </c>
       <c r="I84" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J84">
         <v>15.00956948650922</v>

</xml_diff>